<commit_message>
change in send bulk notification
</commit_message>
<xml_diff>
--- a/docs/API_DEMO.xlsx
+++ b/docs/API_DEMO.xlsx
@@ -3775,7 +3775,7 @@
       </c>
       <c r="I41" s="4" t="inlineStr">
         <is>
-          <t>One item, many targets. Email / SMS / push tokens: "recipients": [...] or a comma-separated "recipient". Push / in-app users: "userIds": [...]. Each target becomes its own notification (own id, status, retry), in order, duplicates dropped; accepted = number of targets. idempotencyKey gets a per-recipient suffix ("key:&lt;hash&gt;"), so repeating the request replays instead of sending twice. At most 500 notifications after expanding. Several recipients and several userIds in one item is a VALIDATION_ERROR; recipients / userIds on POST /v1/notifications (single send) is a VALIDATION_ERROR.</t>
+          <t>One item, many targets. Email / SMS / push tokens: "recipients": [...] or a comma-separated "recipient". Push / in-app users: "userIds": [...]. Each target becomes its own notification (own id, status, retry), in order, duplicates dropped; accepted = number of targets. idempotencyKey gets a per-recipient suffix ("key:&lt;hash&gt;") whenever the list form is used, even with one entry, so repeating the request or adding recipients never re-sends to earlier ones. At most 500 targets listed in total (duplicates included). Several recipients and several userIds in one item is a VALIDATION_ERROR; recipients / userIds on POST /v1/notifications (single send) is a VALIDATION_ERROR.</t>
         </is>
       </c>
       <c r="J41" s="4" t="n"/>
@@ -3797,7 +3797,7 @@
       </c>
       <c r="O41" s="4" t="inlineStr">
         <is>
-          <t>One item, many targets. Email / SMS / push tokens: "recipients": [...] or a comma-separated "recipient". Push / in-app users: "userIds": [...]. Each target becomes its own notification (own id, status, retry), in order, duplicates dropped; accepted = number of targets. idempotencyKey gets a per-recipient suffix ("key:&lt;hash&gt;"), so repeating the request replays instead of sending twice. At most 500 notifications after expanding. Several recipients and several userIds in one item is a VALIDATION_ERROR; recipients / userIds on POST /v1/notifications (single send) is a VALIDATION_ERROR.</t>
+          <t>One item, many targets. Email / SMS / push tokens: "recipients": [...] or a comma-separated "recipient". Push / in-app users: "userIds": [...]. Each target becomes its own notification (own id, status, retry), in order, duplicates dropped; accepted = number of targets. idempotencyKey gets a per-recipient suffix ("key:&lt;hash&gt;") whenever the list form is used, even with one entry, so repeating the request or adding recipients never re-sends to earlier ones. At most 500 targets listed in total (duplicates included). Several recipients and several userIds in one item is a VALIDATION_ERROR; recipients / userIds on POST /v1/notifications (single send) is a VALIDATION_ERROR.</t>
         </is>
       </c>
       <c r="P41" s="7" t="inlineStr">
@@ -11494,7 +11494,7 @@
       </c>
       <c r="I110" s="4" t="inlineStr">
         <is>
-          <t>One item, many targets: recipients (list) or a comma-separated recipient for email/SMS/push tokens, userIds for push/in-app. Each target becomes its own notification (6 here, accepted = 6), in order. The idempotencyKey gets a per-recipient suffix, so repeating the request replays instead of sending twice. Max 500 notifications after expanding.</t>
+          <t>One item, many targets: recipients (list) or a comma-separated recipient for email/SMS/push tokens, userIds for push/in-app. Each target becomes its own notification (6 here, accepted = 6), in order. The idempotencyKey gets a per-recipient suffix, so repeating the request (or adding recipients) replays instead of sending twice. Max 500 targets listed in total.</t>
         </is>
       </c>
       <c r="J110" s="4" t="n"/>

</xml_diff>